<commit_message>
updates to add ev charger replication to robustness
</commit_message>
<xml_diff>
--- a/data/1_assumptions/evs/Record of EV Data Sources.xlsx
+++ b/data/1_assumptions/evs/Record of EV Data Sources.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sarah/Library/CloudStorage/Dropbox-MIT/Regulation/Replication Package/1_assumptions/evs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bcchen\Documents\GitHub\mvpf-climate\data\1_assumptions\evs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B8EF91-F0DA-AB45-8C76-BA7B10BDEA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C1F0AE-A601-4B29-B65E-3D5CB9A36F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{F5A25C02-B73F-D945-B971-D7A4DF68DF8D}"/>
+    <workbookView xWindow="-30460" yWindow="-21880" windowWidth="38620" windowHeight="21100" xr2:uid="{F5A25C02-B73F-D945-B971-D7A4DF68DF8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,16 +27,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>File Name</t>
   </si>
@@ -129,13 +130,19 @@
   </si>
   <si>
     <t>U.S. Census Bureau, Population Division. "Intercensal Estimates of the Resident Population for the United States, Regions, States, and Puerto Rico: April 1, 2000 to July 1, 2010." September 2011.</t>
+  </si>
+  <si>
+    <t>LDV_out_17ihs_I4.dta</t>
+  </si>
+  <si>
+    <t>Cole, Cassandra, Michael Droste, Christopher Knittel, Shanjun Li, and James H. Stock. “Policies for Electrifying the Light-Duty Vehicle Fleet in the United States.” AEA Papers and Proceedings 113 (May 2023): 316–22. https://doi.org/10.1257/pandp.20231063. Replication packet.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -164,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -174,6 +181,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,16 +516,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A191FA47-1611-2449-B9FF-61AD141ABEDC}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="56.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="75.6640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="56.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="75.6328125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -531,7 +539,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -542,7 +550,7 @@
         <v>0.48055555555555557</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="68" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="60">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -556,7 +564,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="30">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -570,7 +578,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="45">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -584,7 +592,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -598,7 +606,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="45">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -612,7 +620,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="45">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -626,7 +634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="45">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -640,7 +648,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="45">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -654,7 +662,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="45">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -668,7 +676,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" ht="45">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -682,7 +690,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="45">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -696,7 +704,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="45">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -710,7 +718,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="45">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -724,7 +732,22 @@
         <v>30</v>
       </c>
     </row>
+    <row r="16" spans="1:4" ht="60">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="1">
+        <v>45945</v>
+      </c>
+      <c r="C16" s="5">
+        <v>0.1423611111111111</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Renamed filepaths for updated table order
</commit_message>
<xml_diff>
--- a/data/1_assumptions/evs/Record of EV Data Sources.xlsx
+++ b/data/1_assumptions/evs/Record of EV Data Sources.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bcchen\Documents\GitHub\mvpf-climate\data\1_assumptions\evs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C1F0AE-A601-4B29-B65E-3D5CB9A36F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF8592E-822E-4A30-9126-68B2E553212C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30460" yWindow="-21880" windowWidth="38620" windowHeight="21100" xr2:uid="{F5A25C02-B73F-D945-B971-D7A4DF68DF8D}"/>
+    <workbookView xWindow="7940" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{F5A25C02-B73F-D945-B971-D7A4DF68DF8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -135,7 +135,7 @@
     <t>LDV_out_17ihs_I4.dta</t>
   </si>
   <si>
-    <t>Cole, Cassandra, Michael Droste, Christopher Knittel, Shanjun Li, and James H. Stock. “Policies for Electrifying the Light-Duty Vehicle Fleet in the United States.” AEA Papers and Proceedings 113 (May 2023): 316–22. https://doi.org/10.1257/pandp.20231063. Replication packet.</t>
+    <t>Cole, Cassandra, Michael Droste, Christopher Knittel, Shanjun Li, and James H. Stock. “Policies for Electrifying the Light-Duty Vehicle Fleet in the United States.” AEA Papers and Proceedings 113 (May 2023): 316–22. https://doi.org/10.1257/pandp.20231063. Replication package.</t>
   </si>
 </sst>
 </file>

</xml_diff>